<commit_message>
update the API documents for main, AI, Detail pages
</commit_message>
<xml_diff>
--- a/메인, AI, 상세 api.xlsx
+++ b/메인, AI, 상세 api.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947ABB2B-3608-44DC-888F-947A935F40A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12600" yWindow="2010" windowWidth="13485" windowHeight="11295"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
   <si>
     <t>메인 페이지</t>
   </si>
@@ -22,6 +23,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>Method</t>
     </r>
@@ -30,6 +35,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>Desc</t>
     </r>
@@ -38,6 +47,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>Request</t>
     </r>
@@ -46,6 +59,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>Response</t>
     </r>
@@ -60,6 +77,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>진행중 행사 중 좋아요순 상위 3개 조회</t>
     </r>
@@ -68,7 +89,7 @@
     <t>{ region: string, status: "ongoing", limit: 3 }</t>
   </si>
   <si>
-    <t>{ success: boolean, region: string, count: number, events: [{ eventId, contentId, title, region, thumbnail, startDate, endDate, likeCount }] }</t>
+    <t>{ success: boolean, region: string, count: number, events: [{ contentId, title, region, thumbnail, startDate, endDate, likeCount }] }</t>
   </si>
   <si>
     <r>
@@ -77,6 +98,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>진행중 행사 중 좋아요순 상위 10개 조회</t>
     </r>
@@ -85,7 +110,7 @@
     <t>{ status: "ongoing", sort: "likeCount", limit: 10 }</t>
   </si>
   <si>
-    <t>{ success: boolean, count: number, events: [{ eventId, contentId, title, region, thumbnail, startDate, endDate, likeCount }] }</t>
+    <t>{ success: boolean, count: number, events: [{ contentId, title, region, thumbnail, startDate, endDate, likeCount }] }</t>
   </si>
   <si>
     <r>
@@ -94,6 +119,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>행사 검색 결과 조회</t>
     </r>
@@ -102,7 +131,7 @@
     <t>{ keyword: string, limit?: number }</t>
   </si>
   <si>
-    <t>{ success: boolean, keyword: string, count: number, events: [{ eventId, contentId, title, region, thumbnail }] }</t>
+    <t>{ success: boolean, keyword: string, count: number, events: [{ eventId, contentId, title, region, thumbnail, startDate, endDate, likeCount }] }</t>
   </si>
   <si>
     <t>AI추천 페이지</t>
@@ -111,6 +140,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>RequestBody</t>
     </r>
@@ -125,19 +158,41 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>지역 + 날짜 + 키워드</t>
     </r>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">를 기반으로, 해당 조건을 만족하는 행사 중 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>관련도 높은 3개 코스를 추천</t>
     </r>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>하고 추천 이유를 반환</t>
     </r>
   </si>
@@ -145,26 +200,21 @@
     <t>{ zipcodeStart: string, zipcodeEnd: string, date: string, keyword: string }</t>
   </si>
   <si>
-    <t>{ success: boolean, zipcodeStart: string, zipcodeEnd: string, date: string, keyword: string, course: [{ eventId, contentId, title, thumbnail, address, description, startDate, endDate }], reason: string }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">로그인한 사용자가 AI가 추천한 행사 3개 코스를 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>내 저장한 추천 목록에 저장</t>
     </r>
   </si>
   <si>
-    <t>{ region: string, date: string, keyword: string, course: [{ eventId: number, order: number }], reason: string }</t>
-  </si>
-  <si>
-    <t>{ success: boolean, message: string, savedCourse: { savedCourseId, userId, region, date, keyword, reason, course: [{ eventId, order }], createdAt } }</t>
-  </si>
-  <si>
     <t>상세 페이지</t>
   </si>
   <si>
@@ -174,6 +224,10 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>상세 정보 전체 조회</t>
     </r>
@@ -182,113 +236,121 @@
     <t>{ eventId: number }</t>
   </si>
   <si>
-    <t>{ success: boolean, event: { contentId, title, thumbnail, images: string[], address, detailAddress, region, startDate, endDate, description, homepage, tel, useTime, fee, organizer, host, latitude, longitude, likeCount, bookmarkCount } }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">해당 행사의 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>좋아요 수 조회</t>
     </r>
   </si>
   <si>
-    <t>{ success: boolean, eventId: number, likeCount: number }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">로그인한 사용자가 해당 행사에 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>좋아요 등록 / 취소(toggle)</t>
     </r>
   </si>
   <si>
-    <t>{ success: boolean, eventId: number, liked: boolean, likeCount: number }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">로그인한 사용자가 해당 행사에 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>좋아요를 눌렀는지 여부 확인</t>
     </r>
   </si>
   <si>
-    <t>{ success: boolean, eventId: number, liked: boolean }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">해당 행사의 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>북마크 수 조회</t>
     </r>
   </si>
   <si>
-    <t>{ success: boolean, eventId: number, bookmarkCount: number }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">로그인한 사용자가 해당 행사에 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>북마크 등록 / 취소(toggle)</t>
     </r>
   </si>
   <si>
-    <t>{ success: boolean, eventId: number, bookmarked: boolean, bookmarkCount: number }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">로그인한 사용자가 해당 행사를 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>북마크했는지 여부 확인</t>
     </r>
   </si>
   <si>
-    <t>{ success: boolean, eventId: number, bookmarked: boolean }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">해당 행사에 등록된 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>댓글 목록 조회</t>
     </r>
   </si>
   <si>
-    <t>{ success: boolean, eventId: number, count: number, comments: [{ commentId, userId, nickname, content, createdAt, updatedAt, isMine }] }</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">로그인한 사용자가 해당 행사에 </t>
     </r>
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>댓글 등록</t>
     </r>
@@ -297,9 +359,6 @@
     <t>{ eventId: number, content: string }</t>
   </si>
   <si>
-    <t>{ success: boolean, message: string, comment: { commentId, eventId, userId, nickname, content, createdAt, updatedAt } }</t>
-  </si>
-  <si>
     <t>PATCH</t>
   </si>
   <si>
@@ -309,51 +368,121 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
       </rPr>
       <t>댓글 수정</t>
     </r>
   </si>
   <si>
     <t>{ commentId: number, content: string }</t>
+  </si>
+  <si>
+    <t>{ success: boolean, course_title: string, region: string, date: string, keyword: string, course: [{ contentId, title, thumbnail, address, startDate, endDate, mapx,mapy }], description: string }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, message: string, savedCourse: { savedCourseId, userId, region, course_title, date, keyword, description, course: [{ contentId, order }], createdAt } }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ region: string, date: string, keyword: string, course_title:string course: [{ contentId: number, order: number }], description: string }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, likeCount: number }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, liked: boolean, likeCount: number }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, liked: boolean }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, bookmarkCount: number }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, bookmarked: boolean, bookmarkCount: number }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, bookmarked: boolean }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, message: string, comment: { commentId, contentId, userId, nickname, content, createdAt, updatedAt } }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, count: number, comments: [{ commentId, userId, nickname, content, createdAt, updatedAt }] }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Response</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, event: { contentId, title, thumbnail, images: string[], address, region,mapx, mapy, startDate, endDate, description, homepage, tel, useTime, fee, organizer, host, latitude, longitude, likeCount, bookmarkCount } }</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
       <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <family val="3"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
       <charset val="129"/>
-      <color theme="1"/>
-      <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -362,16 +491,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF666666"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -379,25 +504,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -728,9 +878,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr defaultRowHeight="16.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.625" customWidth="1"/>
     <col min="2" max="2" width="47.25" customWidth="1"/>
@@ -738,286 +888,332 @@
     <col min="4" max="4" width="69.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" ht="33" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:4" ht="33" customHeight="1">
+      <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="6" spans="1:4">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" ht="49.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:4" ht="49.5" customHeight="1">
+      <c r="A11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="33" customHeight="1">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" ht="33" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="C12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="38.25" customHeight="1">
+      <c r="A20" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="33" customHeight="1">
+      <c r="A22" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="B22" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" ht="38.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="D22" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="33" customHeight="1">
+      <c r="A23" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="4" t="s">
+      <c r="B23" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="C23" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="C24" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="33" customHeight="1">
+      <c r="A25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="33" customHeight="1">
+      <c r="A26" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="B26" s="6" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="22" ht="33" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="C26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A27" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A28" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="B28" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="23" ht="33" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="3" t="s">
+      <c r="C28" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="D28" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A29" s="6" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" s="3" t="s">
+      <c r="B29" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="C29" s="7" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="25" ht="33" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="26" ht="33" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="28" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="29" ht="25.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="D29" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>44</v>
-      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
initiate the frontend  as react(vite) project
</commit_message>
<xml_diff>
--- a/메인, AI, 상세 api.xlsx
+++ b/메인, AI, 상세 api.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947ABB2B-3608-44DC-888F-947A935F40A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF41394-8B5A-4C31-8A30-9FEBB840E246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="87">
   <si>
     <t>메인 페이지</t>
   </si>
@@ -237,7 +237,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">해당 행사의 </t>
+      <t xml:space="preserve">로그인한 사용자가 해당 행사에 </t>
     </r>
     <r>
       <rPr>
@@ -247,7 +247,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>좋아요 수 조회</t>
+      <t>좋아요 등록 / 취소(toggle)</t>
     </r>
   </si>
   <si>
@@ -262,7 +262,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>좋아요 등록 / 취소(toggle)</t>
+      <t>좋아요를 눌렀는지 여부 확인</t>
     </r>
   </si>
   <si>
@@ -277,12 +277,12 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>좋아요를 눌렀는지 여부 확인</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">해당 행사의 </t>
+      <t>북마크 등록 / 취소(toggle)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">로그인한 사용자가 해당 행사를 </t>
     </r>
     <r>
       <rPr>
@@ -292,7 +292,22 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>북마크 수 조회</t>
+      <t>북마크했는지 여부 확인</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">해당 행사에 등록된 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>댓글 목록 조회</t>
     </r>
   </si>
   <si>
@@ -307,12 +322,18 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>북마크 등록 / 취소(toggle)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">로그인한 사용자가 해당 행사를 </t>
+      <t>댓글 등록</t>
+    </r>
+  </si>
+  <si>
+    <t>{ eventId: number, content: string }</t>
+  </si>
+  <si>
+    <t>PATCH</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">로그인한 사용자가 자신이 작성한 </t>
     </r>
     <r>
       <rPr>
@@ -322,12 +343,60 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>북마크했는지 여부 확인</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">해당 행사에 등록된 </t>
+      <t>댓글 수정</t>
+    </r>
+  </si>
+  <si>
+    <t>{ success: boolean, course_title: string, region: string, date: string, keyword: string, course: [{ contentId, title, thumbnail, address, startDate, endDate, mapx,mapy }], description: string }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, message: string, savedCourse: { savedCourseId, userId, region, course_title, date, keyword, description, course: [{ contentId, order }], createdAt } }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ region: string, date: string, keyword: string, course_title:string course: [{ contentId: number, order: number }], description: string }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, liked: boolean, likeCount: number }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, liked: boolean }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, bookmarked: boolean, bookmarkCount: number }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, bookmarked: boolean }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, message: string, comment: { commentId, contentId, userId, nickname, content, createdAt, updatedAt } }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, contentId: number, count: number, comments: [{ commentId, userId, nickname, content, createdAt, updatedAt }] }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Response</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, event: { contentId, title, thumbnail, images: string[], address, region,mapx, mapy, startDate, endDate, description, homepage, tel, useTime, fee, organizer, host, latitude, longitude, likeCount, bookmarkCount } }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>DELETE</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">로그인한 사용자가 자신이 작성한 </t>
     </r>
     <r>
       <rPr>
@@ -337,111 +406,407 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>댓글 목록 조회</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">로그인한 사용자가 해당 행사에 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>댓글 등록</t>
-    </r>
-  </si>
-  <si>
-    <t>{ eventId: number, content: string }</t>
-  </si>
-  <si>
-    <t>PATCH</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">로그인한 사용자가 자신이 작성한 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>댓글 수정</t>
-    </r>
+      <t>댓글 삭제</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
     <t>{ commentId: number, content: string }</t>
-  </si>
-  <si>
-    <t>{ success: boolean, course_title: string, region: string, date: string, keyword: string, course: [{ contentId, title, thumbnail, address, startDate, endDate, mapx,mapy }], description: string }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, message: string, savedCourse: { savedCourseId, userId, region, course_title, date, keyword, description, course: [{ contentId, order }], createdAt } }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ region: string, date: string, keyword: string, course_title:string course: [{ contentId: number, order: number }], description: string }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, contentId: number, likeCount: number }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, contentId: number, liked: boolean, likeCount: number }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, contentId: number, liked: boolean }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, contentId: number, bookmarkCount: number }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, contentId: number, bookmarked: boolean, bookmarkCount: number }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, contentId: number, bookmarked: boolean }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, message: string, comment: { commentId, contentId, userId, nickname, content, createdAt, updatedAt } }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, contentId: number, count: number, comments: [{ commentId, userId, nickname, content, createdAt, updatedAt }] }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Response</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ success: boolean, event: { contentId, title, thumbnail, images: string[], address, region,mapx, mapy, startDate, endDate, description, homepage, tel, useTime, fee, organizer, host, latitude, longitude, likeCount, bookmarkCount } }</t>
-    <phoneticPr fontId="5" type="noConversion"/>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ commentId: number }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ success: boolean, message: string, comment: { commentId, contentId, userId } }</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>로그인 페이지</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Desc</t>
+  </si>
+  <si>
+    <t>사용자가 입력한 이메일 + 비밀번호를 기반으로 회원 정보를 확인하고, 일치하면 로그인 처리 후 사용자 인증 상태를 생성</t>
+  </si>
+  <si>
+    <t>사용자가 입력한 회원 확인 정보를 기반으로 가입된 계정을 조회하고, 일치하는 정보가 있으면 등록된 이메일 정보를 안내</t>
+  </si>
+  <si>
+    <t>PUT</t>
+  </si>
+  <si>
+    <t>사용자가 검색창에 입력한 키워드를 포함한 행사 또는 관광 정보를 조회하여 검색 결과 목록을 반환</t>
+  </si>
+  <si>
+    <t>마이페이지</t>
+  </si>
+  <si>
+    <t>로그인한 사용자의 닉네임, 이메일 등 마이페이지에 표시될 회원 정보 전체를 조회</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로그인한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>사용자가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>닉네임</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이메일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>회원</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수정하면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>변경된</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>내용을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기존</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>회원</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>반영</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>로그인한 사용자가 메인/상세 페이지에서 저장한 북마크 행사 목록 전체를 조회하고, 각 항목의 북마크 상태가 유지된 데이터를 반환</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>로그인한 사용자가 마이페이지의 북마크 목록에서 특정 행사의 북마크를 해제하면, 해당 북마크 데이터를 삭제하고 새로고침 시목록에서 제거된 상태로 반영</t>
+  </si>
+  <si>
+    <t>로그인한 사용자가 이전에 저장한 AI 추천 코스 목록 전체를 조회하여 마이페이지에 표시</t>
+  </si>
+  <si>
+    <t>로그인한 사용자가 저장된 AI 추천 코스 중 선택한 코스중 삭제버튼을 누르면, 해당 추천 코스 데이터를 제거하고 목록에서 제외</t>
+  </si>
+  <si>
+    <t>회원가입 페이지</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>API 종류</t>
+  </si>
+  <si>
+    <t>메서드</t>
+  </si>
+  <si>
+    <t>설명</t>
+  </si>
+  <si>
+    <t>회원가입</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>사용자가 이메일, 비밀번호, 닉네임으로 회원가입한다. 기본 프로필 이미지도 함께 설정될 수 있다.</t>
+  </si>
+  <si>
+    <t>닉네임 중복확인</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>GET</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>사용자의 닉네임을 DB에 있는 닉네임들과 비교하여 중복된 값이 없으면 중복된 값이 없다는 메시지를 띄우며 진행, 있으면 중복된 값이 있다는 메시지를 띄우며 진행불가 처리</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>이메일 중복확인</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>사용자의 이메일을 DB에 있는 이메일들과 비교하여 중복된 값이 없으면 중복된 값이 없다는 메시지를 띄우며 진행, 있으면 중복된 값이 있다는 메시지를 띄우며 진행불가 처리</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>목록 페이지</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>API 종류</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>전체 행사 목록 조회</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>전체 행사 목록을 조회한다. 목록 페이지의 기본 데이터가 된다.</t>
+  </si>
+  <si>
+    <t>행사 필터 조회</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>지역, 상태, 카테고리, 날짜 등 여러 조건을 조합해 행사 목록을 조회한다.</t>
+  </si>
+  <si>
+    <t>전체 카테고리 목록 조회</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>행사 분류 카테고리 목록을 조회한다.</t>
+  </si>
+  <si>
+    <t>지역별 하위 구역 목록 조회</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>필요 시 시군구 등 세부 지역 목록을 조회한다.</t>
+  </si>
+  <si>
+    <t>자동완성 검색</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>행사명 검색 시 자동완성 목록을 제공한다.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -481,8 +846,65 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF181818"/>
+      <name val="&quot;Apple SD Gothic Neo&quot;"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Apple SD Gothic Neo&quot;"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Apple SD Gothic Neo&quot;"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -495,8 +917,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD1E5F5"/>
+        <bgColor rgb="FFD1E5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE5EFF6"/>
+        <bgColor rgb="FFE5EFF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -519,30 +959,229 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF9A9A9A"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF3E3E3E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA8A8A8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF9A9A9A"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF3E3E3E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA8A8A8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA8A8A8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA8A8A8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA8A8A8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA8A8A8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -879,7 +1518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.625" customWidth="1"/>
@@ -1003,7 +1642,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="33" customHeight="1">
@@ -1014,10 +1653,10 @@
         <v>20</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="16.5" customHeight="1">
@@ -1069,7 +1708,7 @@
         <v>16</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="38.25" customHeight="1">
@@ -1083,12 +1722,12 @@
         <v>23</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="33">
       <c r="A21" s="6" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>24</v>
@@ -1097,12 +1736,12 @@
         <v>23</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="33" customHeight="1">
       <c r="A22" s="6" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>25</v>
@@ -1111,12 +1750,12 @@
         <v>23</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="33" customHeight="1">
       <c r="A23" s="6" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>26</v>
@@ -1125,10 +1764,10 @@
         <v>23</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="33">
       <c r="A24" s="6" t="s">
         <v>5</v>
       </c>
@@ -1139,12 +1778,12 @@
         <v>23</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="33" customHeight="1">
       <c r="A25" s="6" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>28</v>
@@ -1153,67 +1792,287 @@
         <v>23</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="33" customHeight="1">
       <c r="A26" s="6" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>29</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="25.5" customHeight="1">
       <c r="A27" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A28" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="25.5" customHeight="1" thickBot="1"/>
+    <row r="30" spans="1:4" ht="41.25" customHeight="1">
+      <c r="A30" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="12"/>
+    </row>
+    <row r="31" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A31" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A32" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A33" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A34" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="25.5" customHeight="1">
-      <c r="A28" s="6" t="s">
+      <c r="B34" s="15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="16.5" customHeight="1" thickBot="1"/>
+    <row r="37" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A37" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="12"/>
+    </row>
+    <row r="38" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A38" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A39" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A40" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A41" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A42" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A43" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A44" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="16.5" customHeight="1" thickBot="1"/>
+    <row r="47" spans="1:3" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A47" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" s="18"/>
+      <c r="C47" s="19"/>
+    </row>
+    <row r="48" spans="1:3" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A48" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A49" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="B49" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="25.5" customHeight="1">
-      <c r="A29" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>45</v>
+      <c r="C49" s="21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A50" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B50" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C50" s="23" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A51" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="B51" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="C51" s="24" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="16.5" customHeight="1" thickBot="1"/>
+    <row r="54" spans="1:3" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A54" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="B54" s="26"/>
+      <c r="C54" s="27"/>
+    </row>
+    <row r="55" spans="1:3" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A55" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55" s="20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A56" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="B56" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" s="22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A57" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B57" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57" s="22" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A58" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B58" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" s="22" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A59" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="B59" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C59" s="22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A60" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B60" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C60" s="24" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <mergeCells count="4">
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A54:C54"/>
+  </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>